<commit_message>
Structure v0.2 : suivi de stock par mouvement, reports de ventes, forçages, points, scénarios
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/ENTREE_COMMANDES_FOURN.xlsx
+++ b/modeles/xlsx/ENTREE_COMMANDES_FOURN.xlsx
@@ -50,13 +50,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="14" max="14" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -67,37 +73,67 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Code fournisseur</t>
+          <t xml:space="preserve">N commande vente associee</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Code produit</t>
+          <t xml:space="preserve">Code fournisseur</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Plateforme</t>
+          <t xml:space="preserve">Nom fournisseur</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Date commande</t>
+          <t xml:space="preserve">Societe partenaire</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Date livraison prevue</t>
+          <t xml:space="preserve">Code produit</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Quantite</t>
+          <t xml:space="preserve">Code point</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Statut</t>
+          <t xml:space="preserve">Date commande</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Date limite livraison</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Etat</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Quantite commandee</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Quantite receptionnee</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Quantite reste a livrer</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Prix unitaire</t>
         </is>
       </c>
     </row>

</xml_diff>